<commit_message>
Fix city locator (title-based) across 4 pages; CarePlan/Charts direct city; runners honor code:2 popup soft-skip
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/CarePlan/LSTP_CarePlan_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/CarePlan/LSTP_CarePlan_WF001.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrishnan6\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\CarePlan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FECDC7-E469-4D85-B9CE-72DE925BD973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B1FABB-377E-42EE-B8B7-5D8FE9A8B2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{33E707BA-C33D-4108-BB34-C72B89CD78DB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="370">
   <si>
     <t>StepNo</t>
   </si>
@@ -185,15 +185,9 @@
     <t>POSTALCODE</t>
   </si>
   <si>
-    <t>Click Find to resolve address from postal code</t>
-  </si>
-  <si>
     <t>Wait for address lookup results</t>
   </si>
   <si>
-    <t>Select address row from lookup results</t>
-  </si>
-  <si>
     <t>tbl_SelectRow</t>
   </si>
   <si>
@@ -1149,6 +1143,12 @@
   </si>
   <si>
     <t>pageSearchPatient</t>
+  </si>
+  <si>
+    <t>// Click Find to resolve address from postal code</t>
+  </si>
+  <si>
+    <t>// Select address row from lookup results</t>
   </si>
 </sst>
 </file>
@@ -1676,13 +1676,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C7" t="s">
         <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="F7" t="s">
         <v>23</v>
@@ -1730,7 +1730,7 @@
         <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D10" t="s">
         <v>34</v>
@@ -1849,7 +1849,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>368</v>
       </c>
       <c r="C17" t="s">
         <v>40</v>
@@ -1866,7 +1866,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C18" t="s">
         <v>40</v>
@@ -1880,13 +1880,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>369</v>
       </c>
       <c r="C19" t="s">
         <v>40</v>
       </c>
       <c r="D19" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F19" t="s">
         <v>23</v>
@@ -1897,19 +1897,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C20" t="s">
         <v>40</v>
       </c>
       <c r="D20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F20" t="s">
         <v>31</v>
       </c>
+      <c r="J20" t="s">
+        <v>284</v>
+      </c>
       <c r="K20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -1917,19 +1920,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C21" t="s">
         <v>40</v>
       </c>
       <c r="D21" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" t="s">
+        <v>55</v>
+      </c>
+      <c r="K21" t="s">
         <v>56</v>
-      </c>
-      <c r="F21" t="s">
-        <v>57</v>
-      </c>
-      <c r="K21" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -1937,19 +1940,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C22" t="s">
         <v>40</v>
       </c>
       <c r="D22" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F22" t="s">
         <v>31</v>
       </c>
       <c r="K22" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -1957,19 +1960,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
         <v>40</v>
       </c>
       <c r="D23" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F23" t="s">
         <v>31</v>
       </c>
       <c r="K23" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -1977,19 +1980,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C24" t="s">
         <v>40</v>
       </c>
       <c r="D24" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F24" t="s">
         <v>31</v>
       </c>
       <c r="K24" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -1997,13 +2000,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C25" t="s">
         <v>40</v>
       </c>
       <c r="D25" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F25" t="s">
         <v>23</v>
@@ -2014,7 +2017,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C26" t="s">
         <v>40</v>
@@ -2028,19 +2031,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C27" t="s">
         <v>40</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F27" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K27" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -2048,19 +2051,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C28" t="s">
         <v>40</v>
       </c>
       <c r="D28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F28" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K28" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -2068,19 +2071,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C29" t="s">
         <v>40</v>
       </c>
       <c r="D29" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F29" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K29" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -2088,19 +2091,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C30" t="s">
         <v>40</v>
       </c>
       <c r="D30" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F30" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K30" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -2108,19 +2111,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C31" t="s">
         <v>40</v>
       </c>
       <c r="D31" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F31" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K31" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -2128,19 +2131,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C32" t="s">
         <v>40</v>
       </c>
       <c r="D32" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F32" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K32" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -2148,13 +2151,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C33" t="s">
         <v>40</v>
       </c>
       <c r="D33" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F33" t="s">
         <v>23</v>
@@ -2165,10 +2168,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C34" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F34" t="s">
         <v>20</v>
@@ -2179,19 +2182,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35" t="s">
+        <v>90</v>
+      </c>
+      <c r="D35" t="s">
+        <v>92</v>
+      </c>
+      <c r="F35" t="s">
         <v>93</v>
       </c>
-      <c r="C35" t="s">
-        <v>92</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="J35" t="s">
         <v>94</v>
-      </c>
-      <c r="F35" t="s">
-        <v>95</v>
-      </c>
-      <c r="J35" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -2199,22 +2202,22 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
+        <v>95</v>
+      </c>
+      <c r="C36" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36" t="s">
+        <v>92</v>
+      </c>
+      <c r="F36" t="s">
+        <v>96</v>
+      </c>
+      <c r="G36" t="s">
         <v>97</v>
       </c>
-      <c r="C36" t="s">
-        <v>92</v>
-      </c>
-      <c r="D36" t="s">
-        <v>94</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="H36" t="s">
         <v>98</v>
-      </c>
-      <c r="G36" t="s">
-        <v>99</v>
-      </c>
-      <c r="H36" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -2222,13 +2225,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D37" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F37" t="s">
         <v>23</v>
@@ -2239,7 +2242,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C38" t="s">
         <v>19</v>
@@ -2253,13 +2256,13 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C39" t="s">
         <v>19</v>
       </c>
       <c r="D39" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F39" t="s">
         <v>23</v>
@@ -2270,7 +2273,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C40" t="s">
         <v>29</v>
@@ -2284,7 +2287,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C41" t="s">
         <v>29</v>
@@ -2335,13 +2338,13 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>106</v>
+      </c>
+      <c r="C44" t="s">
+        <v>107</v>
+      </c>
+      <c r="D44" t="s">
         <v>108</v>
-      </c>
-      <c r="C44" t="s">
-        <v>109</v>
-      </c>
-      <c r="D44" t="s">
-        <v>110</v>
       </c>
       <c r="F44" t="s">
         <v>23</v>
@@ -2352,10 +2355,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C45" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F45" t="s">
         <v>20</v>
@@ -2366,22 +2369,22 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
+        <v>111</v>
+      </c>
+      <c r="C46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D46" t="s">
+        <v>112</v>
+      </c>
+      <c r="F46" t="s">
+        <v>96</v>
+      </c>
+      <c r="G46" t="s">
         <v>113</v>
       </c>
-      <c r="C46" t="s">
-        <v>112</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="H46" t="s">
         <v>114</v>
-      </c>
-      <c r="F46" t="s">
-        <v>98</v>
-      </c>
-      <c r="G46" t="s">
-        <v>115</v>
-      </c>
-      <c r="H46" t="s">
-        <v>116</v>
       </c>
       <c r="J46" t="b">
         <v>1</v>
@@ -2392,19 +2395,19 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C47" t="s">
+        <v>110</v>
+      </c>
+      <c r="D47" t="s">
         <v>112</v>
       </c>
-      <c r="D47" t="s">
-        <v>114</v>
-      </c>
       <c r="F47" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J47" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
@@ -2412,13 +2415,13 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C48" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D48" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F48" t="s">
         <v>23</v>
@@ -2429,10 +2432,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C49" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F49" t="s">
         <v>20</v>
@@ -2443,13 +2446,13 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C50" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D50" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F50" t="s">
         <v>23</v>
@@ -2460,10 +2463,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C51" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F51" t="s">
         <v>20</v>
@@ -2474,19 +2477,19 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
+        <v>124</v>
+      </c>
+      <c r="C52" t="s">
+        <v>123</v>
+      </c>
+      <c r="D52" t="s">
+        <v>125</v>
+      </c>
+      <c r="F52" t="s">
+        <v>55</v>
+      </c>
+      <c r="K52" t="s">
         <v>126</v>
-      </c>
-      <c r="C52" t="s">
-        <v>125</v>
-      </c>
-      <c r="D52" t="s">
-        <v>127</v>
-      </c>
-      <c r="F52" t="s">
-        <v>57</v>
-      </c>
-      <c r="K52" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
@@ -2494,19 +2497,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
+        <v>127</v>
+      </c>
+      <c r="C53" t="s">
+        <v>123</v>
+      </c>
+      <c r="D53" t="s">
+        <v>128</v>
+      </c>
+      <c r="F53" t="s">
+        <v>55</v>
+      </c>
+      <c r="K53" t="s">
         <v>129</v>
-      </c>
-      <c r="C53" t="s">
-        <v>125</v>
-      </c>
-      <c r="D53" t="s">
-        <v>130</v>
-      </c>
-      <c r="F53" t="s">
-        <v>57</v>
-      </c>
-      <c r="K53" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -2514,19 +2517,19 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
+        <v>130</v>
+      </c>
+      <c r="C54" t="s">
+        <v>123</v>
+      </c>
+      <c r="D54" t="s">
+        <v>131</v>
+      </c>
+      <c r="F54" t="s">
+        <v>55</v>
+      </c>
+      <c r="K54" t="s">
         <v>132</v>
-      </c>
-      <c r="C54" t="s">
-        <v>125</v>
-      </c>
-      <c r="D54" t="s">
-        <v>133</v>
-      </c>
-      <c r="F54" t="s">
-        <v>57</v>
-      </c>
-      <c r="K54" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
@@ -2534,19 +2537,19 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
+        <v>133</v>
+      </c>
+      <c r="C55" t="s">
+        <v>123</v>
+      </c>
+      <c r="D55" t="s">
+        <v>134</v>
+      </c>
+      <c r="F55" t="s">
+        <v>55</v>
+      </c>
+      <c r="K55" t="s">
         <v>135</v>
-      </c>
-      <c r="C55" t="s">
-        <v>125</v>
-      </c>
-      <c r="D55" t="s">
-        <v>136</v>
-      </c>
-      <c r="F55" t="s">
-        <v>57</v>
-      </c>
-      <c r="K55" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -2554,13 +2557,13 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C56" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D56" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F56" t="s">
         <v>23</v>
@@ -2571,10 +2574,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C57" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F57" t="s">
         <v>20</v>
@@ -2585,22 +2588,22 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C58" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D58" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F58" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G58" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H58" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J58" t="b">
         <v>1</v>
@@ -2611,10 +2614,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F59" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J59">
         <v>1</v>
@@ -2625,13 +2628,13 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C60" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D60" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F60" t="s">
         <v>23</v>
@@ -2642,13 +2645,13 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C61" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D61" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F61" t="s">
         <v>23</v>
@@ -2659,10 +2662,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C62" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F62" t="s">
         <v>20</v>
@@ -2673,19 +2676,19 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
+        <v>148</v>
+      </c>
+      <c r="C63" t="s">
+        <v>147</v>
+      </c>
+      <c r="D63" t="s">
+        <v>149</v>
+      </c>
+      <c r="F63" t="s">
+        <v>55</v>
+      </c>
+      <c r="K63" t="s">
         <v>150</v>
-      </c>
-      <c r="C63" t="s">
-        <v>149</v>
-      </c>
-      <c r="D63" t="s">
-        <v>151</v>
-      </c>
-      <c r="F63" t="s">
-        <v>57</v>
-      </c>
-      <c r="K63" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
@@ -2693,19 +2696,19 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
+        <v>151</v>
+      </c>
+      <c r="C64" t="s">
+        <v>147</v>
+      </c>
+      <c r="D64" t="s">
+        <v>152</v>
+      </c>
+      <c r="F64" t="s">
+        <v>55</v>
+      </c>
+      <c r="K64" t="s">
         <v>153</v>
-      </c>
-      <c r="C64" t="s">
-        <v>149</v>
-      </c>
-      <c r="D64" t="s">
-        <v>154</v>
-      </c>
-      <c r="F64" t="s">
-        <v>57</v>
-      </c>
-      <c r="K64" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
@@ -2713,19 +2716,19 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
+        <v>154</v>
+      </c>
+      <c r="C65" t="s">
+        <v>147</v>
+      </c>
+      <c r="D65" t="s">
+        <v>155</v>
+      </c>
+      <c r="F65" t="s">
+        <v>55</v>
+      </c>
+      <c r="K65" t="s">
         <v>156</v>
-      </c>
-      <c r="C65" t="s">
-        <v>149</v>
-      </c>
-      <c r="D65" t="s">
-        <v>157</v>
-      </c>
-      <c r="F65" t="s">
-        <v>57</v>
-      </c>
-      <c r="K65" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
@@ -2733,19 +2736,19 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
+        <v>157</v>
+      </c>
+      <c r="C66" t="s">
+        <v>147</v>
+      </c>
+      <c r="D66" t="s">
+        <v>158</v>
+      </c>
+      <c r="F66" t="s">
+        <v>55</v>
+      </c>
+      <c r="K66" t="s">
         <v>159</v>
-      </c>
-      <c r="C66" t="s">
-        <v>149</v>
-      </c>
-      <c r="D66" t="s">
-        <v>160</v>
-      </c>
-      <c r="F66" t="s">
-        <v>57</v>
-      </c>
-      <c r="K66" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -2753,13 +2756,13 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C67" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D67" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F67" t="s">
         <v>23</v>
@@ -2770,10 +2773,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C68" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F68" t="s">
         <v>20</v>
@@ -2784,13 +2787,13 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C69" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D69" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F69" t="s">
         <v>23</v>
@@ -2801,10 +2804,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C70" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F70" t="s">
         <v>20</v>
@@ -2815,22 +2818,22 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C71" t="s">
+        <v>110</v>
+      </c>
+      <c r="D71" t="s">
         <v>112</v>
       </c>
-      <c r="D71" t="s">
+      <c r="F71" t="s">
+        <v>96</v>
+      </c>
+      <c r="G71" t="s">
+        <v>113</v>
+      </c>
+      <c r="H71" t="s">
         <v>114</v>
-      </c>
-      <c r="F71" t="s">
-        <v>98</v>
-      </c>
-      <c r="G71" t="s">
-        <v>115</v>
-      </c>
-      <c r="H71" t="s">
-        <v>116</v>
       </c>
       <c r="J71" t="b">
         <v>1</v>
@@ -2841,10 +2844,10 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F72" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J72">
         <v>1</v>
@@ -2855,13 +2858,13 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C73" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D73" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F73" t="s">
         <v>23</v>
@@ -2872,10 +2875,10 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C74" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F74" t="s">
         <v>20</v>
@@ -2886,22 +2889,22 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C75" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D75" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F75" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G75" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H75" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J75" t="b">
         <v>1</v>
@@ -2912,10 +2915,10 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F76" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J76">
         <v>1</v>
@@ -2926,13 +2929,13 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C77" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D77" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F77" t="s">
         <v>23</v>
@@ -2943,10 +2946,10 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C78" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F78" t="s">
         <v>20</v>
@@ -2957,19 +2960,19 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C79" t="s">
+        <v>175</v>
+      </c>
+      <c r="D79" t="s">
         <v>177</v>
-      </c>
-      <c r="D79" t="s">
-        <v>179</v>
       </c>
       <c r="F79" t="s">
         <v>31</v>
       </c>
       <c r="K79" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -2977,10 +2980,10 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C80" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D80" t="s">
         <v>34</v>
@@ -2994,10 +2997,10 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C81" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F81" t="s">
         <v>20</v>
@@ -3008,13 +3011,13 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C82" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D82" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F82" t="s">
         <v>23</v>
@@ -3025,10 +3028,10 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C83" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F83" t="s">
         <v>20</v>
@@ -3039,13 +3042,13 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C84" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D84" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F84" t="s">
         <v>23</v>
@@ -3056,10 +3059,10 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C85" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F85" t="s">
         <v>20</v>
@@ -3070,13 +3073,13 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C86" t="s">
+        <v>187</v>
+      </c>
+      <c r="D86" t="s">
         <v>189</v>
-      </c>
-      <c r="D86" t="s">
-        <v>191</v>
       </c>
       <c r="F86" t="s">
         <v>23</v>
@@ -3087,13 +3090,13 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C87" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D87" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F87" t="s">
         <v>23</v>
@@ -3104,10 +3107,10 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C88" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F88" t="s">
         <v>20</v>
@@ -3118,10 +3121,10 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F89" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J89">
         <v>1</v>
@@ -3132,22 +3135,22 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C90" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D90" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F90" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G90" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H90" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J90" t="b">
         <v>1</v>
@@ -3158,22 +3161,22 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C91" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D91" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F91" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G91" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H91" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J91" t="b">
         <v>1</v>
@@ -3184,10 +3187,10 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F92" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J92">
         <v>1</v>
@@ -3198,13 +3201,13 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C93" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D93" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F93" t="s">
         <v>23</v>
@@ -3215,13 +3218,13 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C94" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D94" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F94" t="s">
         <v>23</v>
@@ -3232,10 +3235,10 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C95" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F95" t="s">
         <v>20</v>
@@ -3246,19 +3249,19 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
+        <v>202</v>
+      </c>
+      <c r="C96" t="s">
+        <v>201</v>
+      </c>
+      <c r="D96" t="s">
+        <v>203</v>
+      </c>
+      <c r="F96" t="s">
+        <v>55</v>
+      </c>
+      <c r="K96" t="s">
         <v>204</v>
-      </c>
-      <c r="C96" t="s">
-        <v>203</v>
-      </c>
-      <c r="D96" t="s">
-        <v>205</v>
-      </c>
-      <c r="F96" t="s">
-        <v>57</v>
-      </c>
-      <c r="K96" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.25">
@@ -3266,10 +3269,10 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C97" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F97" t="s">
         <v>20</v>
@@ -3280,13 +3283,13 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C98" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D98" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F98" t="s">
         <v>23</v>
@@ -3297,10 +3300,10 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C99" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F99" t="s">
         <v>20</v>
@@ -3311,13 +3314,13 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C100" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D100" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F100" t="s">
         <v>23</v>
@@ -3328,13 +3331,13 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C101" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D101" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F101" t="s">
         <v>23</v>
@@ -3345,10 +3348,10 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C102" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F102" t="s">
         <v>20</v>
@@ -3359,10 +3362,10 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F103" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J103">
         <v>1</v>
@@ -3373,22 +3376,22 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C104" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D104" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F104" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G104" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H104" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J104" t="b">
         <v>1</v>
@@ -3399,22 +3402,22 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C105" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D105" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F105" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G105" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H105" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J105" t="b">
         <v>1</v>
@@ -3425,10 +3428,10 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F106" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J106">
         <v>1</v>
@@ -3439,13 +3442,13 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C107" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D107" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F107" t="s">
         <v>23</v>
@@ -3456,13 +3459,13 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C108" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D108" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F108" t="s">
         <v>23</v>
@@ -3473,10 +3476,10 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C109" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F109" t="s">
         <v>20</v>
@@ -3487,19 +3490,19 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C110" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D110" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="F110" t="s">
         <v>31</v>
       </c>
       <c r="K110" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.25">
@@ -3507,10 +3510,10 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C111" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F111" t="s">
         <v>20</v>
@@ -3521,13 +3524,13 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C112" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D112" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F112" t="s">
         <v>23</v>
@@ -3538,10 +3541,10 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C113" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F113" t="s">
         <v>20</v>
@@ -3552,13 +3555,13 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C114" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D114" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F114" t="s">
         <v>23</v>
@@ -3569,10 +3572,10 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C115" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F115" t="s">
         <v>20</v>
@@ -3583,10 +3586,10 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F116" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J116">
         <v>1</v>
@@ -3597,22 +3600,22 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C117" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D117" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F117" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G117" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H117" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J117" t="b">
         <v>1</v>
@@ -3623,22 +3626,22 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C118" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D118" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F118" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G118" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H118" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J118" t="b">
         <v>1</v>
@@ -3649,10 +3652,10 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F119" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J119">
         <v>1</v>
@@ -3663,13 +3666,13 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C120" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D120" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F120" t="s">
         <v>23</v>
@@ -3680,13 +3683,13 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C121" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D121" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F121" t="s">
         <v>23</v>
@@ -3697,10 +3700,10 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C122" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="F122" t="s">
         <v>20</v>
@@ -3711,19 +3714,19 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
+        <v>237</v>
+      </c>
+      <c r="C123" t="s">
+        <v>236</v>
+      </c>
+      <c r="D123" t="s">
+        <v>238</v>
+      </c>
+      <c r="F123" t="s">
+        <v>55</v>
+      </c>
+      <c r="K123" t="s">
         <v>239</v>
-      </c>
-      <c r="C123" t="s">
-        <v>238</v>
-      </c>
-      <c r="D123" t="s">
-        <v>240</v>
-      </c>
-      <c r="F123" t="s">
-        <v>57</v>
-      </c>
-      <c r="K123" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
@@ -3731,10 +3734,10 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C124" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F124" t="s">
         <v>20</v>
@@ -3745,13 +3748,13 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C125" t="s">
+        <v>241</v>
+      </c>
+      <c r="D125" t="s">
         <v>243</v>
-      </c>
-      <c r="D125" t="s">
-        <v>245</v>
       </c>
       <c r="F125" t="s">
         <v>23</v>
@@ -3762,10 +3765,10 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C126" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F126" t="s">
         <v>20</v>
@@ -3776,10 +3779,10 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F127" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J127">
         <v>1</v>
@@ -3790,22 +3793,22 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C128" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D128" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F128" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G128" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H128" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J128" t="b">
         <v>1</v>
@@ -3816,22 +3819,22 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C129" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D129" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F129" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G129" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H129" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J129" t="b">
         <v>1</v>
@@ -3842,10 +3845,10 @@
         <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="F130" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J130">
         <v>1</v>
@@ -3856,13 +3859,13 @@
         <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C131" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D131" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F131" t="s">
         <v>23</v>
@@ -3873,13 +3876,13 @@
         <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C132" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D132" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F132" t="s">
         <v>23</v>
@@ -3890,10 +3893,10 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C133" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="F133" t="s">
         <v>20</v>
@@ -3904,19 +3907,19 @@
         <v>133</v>
       </c>
       <c r="B134" t="s">
+        <v>250</v>
+      </c>
+      <c r="C134" t="s">
+        <v>236</v>
+      </c>
+      <c r="D134" t="s">
+        <v>251</v>
+      </c>
+      <c r="F134" t="s">
+        <v>55</v>
+      </c>
+      <c r="K134" t="s">
         <v>252</v>
-      </c>
-      <c r="C134" t="s">
-        <v>238</v>
-      </c>
-      <c r="D134" t="s">
-        <v>253</v>
-      </c>
-      <c r="F134" t="s">
-        <v>57</v>
-      </c>
-      <c r="K134" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.25">
@@ -3924,10 +3927,10 @@
         <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C135" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F135" t="s">
         <v>20</v>
@@ -3938,13 +3941,13 @@
         <v>135</v>
       </c>
       <c r="B136" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C136" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D136" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="F136" t="s">
         <v>23</v>
@@ -3955,10 +3958,10 @@
         <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C137" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F137" t="s">
         <v>20</v>
@@ -3969,10 +3972,10 @@
         <v>137</v>
       </c>
       <c r="B138" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="F138" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J138">
         <v>1</v>
@@ -3983,22 +3986,22 @@
         <v>138</v>
       </c>
       <c r="B139" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C139" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D139" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F139" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G139" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H139" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J139" t="b">
         <v>1</v>
@@ -4009,22 +4012,22 @@
         <v>139</v>
       </c>
       <c r="B140" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C140" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D140" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F140" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G140" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H140" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J140" t="b">
         <v>1</v>
@@ -4035,10 +4038,10 @@
         <v>140</v>
       </c>
       <c r="B141" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F141" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J141">
         <v>1</v>
@@ -4049,13 +4052,13 @@
         <v>141</v>
       </c>
       <c r="B142" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C142" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D142" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F142" t="s">
         <v>23</v>
@@ -4066,13 +4069,13 @@
         <v>142</v>
       </c>
       <c r="B143" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C143" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D143" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F143" t="s">
         <v>23</v>
@@ -4083,10 +4086,10 @@
         <v>143</v>
       </c>
       <c r="B144" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C144" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="F144" t="s">
         <v>20</v>
@@ -4097,19 +4100,19 @@
         <v>144</v>
       </c>
       <c r="B145" t="s">
+        <v>261</v>
+      </c>
+      <c r="C145" t="s">
+        <v>236</v>
+      </c>
+      <c r="D145" t="s">
+        <v>262</v>
+      </c>
+      <c r="F145" t="s">
+        <v>55</v>
+      </c>
+      <c r="K145" t="s">
         <v>263</v>
-      </c>
-      <c r="C145" t="s">
-        <v>238</v>
-      </c>
-      <c r="D145" t="s">
-        <v>264</v>
-      </c>
-      <c r="F145" t="s">
-        <v>57</v>
-      </c>
-      <c r="K145" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="146" spans="1:11" x14ac:dyDescent="0.25">
@@ -4117,10 +4120,10 @@
         <v>145</v>
       </c>
       <c r="B146" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C146" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F146" t="s">
         <v>20</v>
@@ -4131,13 +4134,13 @@
         <v>146</v>
       </c>
       <c r="B147" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C147" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D147" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="F147" t="s">
         <v>23</v>
@@ -4148,10 +4151,10 @@
         <v>147</v>
       </c>
       <c r="B148" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C148" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F148" t="s">
         <v>20</v>
@@ -4162,10 +4165,10 @@
         <v>148</v>
       </c>
       <c r="B149" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F149" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J149">
         <v>1</v>
@@ -4176,22 +4179,22 @@
         <v>149</v>
       </c>
       <c r="B150" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C150" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D150" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F150" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G150" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H150" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J150" t="b">
         <v>1</v>
@@ -4202,22 +4205,22 @@
         <v>150</v>
       </c>
       <c r="B151" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C151" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D151" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F151" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G151" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H151" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J151" t="b">
         <v>1</v>
@@ -4228,13 +4231,13 @@
         <v>151</v>
       </c>
       <c r="B152" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C152" t="s">
         <v>19</v>
       </c>
       <c r="D152" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F152" t="s">
         <v>23</v>
@@ -4245,13 +4248,13 @@
         <v>152</v>
       </c>
       <c r="B153" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C153" t="s">
         <v>19</v>
       </c>
       <c r="D153" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F153" t="s">
         <v>23</v>
@@ -4262,10 +4265,10 @@
         <v>153</v>
       </c>
       <c r="B154" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F154" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J154">
         <v>3</v>
@@ -4289,16 +4292,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>278</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -4306,13 +4309,13 @@
         <v>43</v>
       </c>
       <c r="B2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C2" t="s">
+        <v>280</v>
+      </c>
+      <c r="D2" t="s">
         <v>281</v>
-      </c>
-      <c r="C2" t="s">
-        <v>282</v>
-      </c>
-      <c r="D2" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -4320,363 +4323,363 @@
         <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C3" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D3" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D4" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C6">
         <v>2071234567</v>
       </c>
       <c r="D6" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C7">
         <v>7712345678</v>
       </c>
       <c r="D7" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C8" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D8" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C9" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D9" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B10" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C10" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D10" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B11" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C11" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D11" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B12" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C12" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D12" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B13" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C13" t="s">
+        <v>297</v>
+      </c>
+      <c r="D13" t="s">
         <v>299</v>
-      </c>
-      <c r="D13" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C14" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="D14" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B15" t="s">
+        <v>302</v>
+      </c>
+      <c r="C15" t="s">
+        <v>303</v>
+      </c>
+      <c r="D15" t="s">
         <v>304</v>
-      </c>
-      <c r="C15" t="s">
-        <v>305</v>
-      </c>
-      <c r="D15" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B16" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C16" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D16" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B17" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C17" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D17" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B18" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C18" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D18" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B19" t="s">
+        <v>311</v>
+      </c>
+      <c r="C19" t="s">
+        <v>312</v>
+      </c>
+      <c r="D19" t="s">
         <v>313</v>
-      </c>
-      <c r="C19" t="s">
-        <v>314</v>
-      </c>
-      <c r="D19" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B20" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C20" t="s">
+        <v>312</v>
+      </c>
+      <c r="D20" t="s">
         <v>314</v>
-      </c>
-      <c r="D20" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B21" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C21" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D21" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B22" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C22" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D22" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B23" t="s">
+        <v>318</v>
+      </c>
+      <c r="C23" t="s">
+        <v>319</v>
+      </c>
+      <c r="D23" t="s">
         <v>320</v>
-      </c>
-      <c r="C23" t="s">
-        <v>321</v>
-      </c>
-      <c r="D23" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B24" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C24" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D24" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B25" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C25" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D25" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B26" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C26" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D26" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B27" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C27" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D27" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B28" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C28" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D28" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
   </sheetData>
@@ -4695,71 +4698,71 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B9" s="2">
         <v>152</v>
@@ -4767,7 +4770,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B10" s="2">
         <v>20</v>
@@ -4775,7 +4778,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B11" s="2">
         <v>57</v>
@@ -4783,15 +4786,15 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B13" s="3">
         <v>46146</v>
@@ -4799,7 +4802,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B14" s="3">
         <v>46146</v>
@@ -4807,31 +4810,31 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B18" s="2">
         <v>17</v>
@@ -4839,18 +4842,18 @@
     </row>
     <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
   </sheetData>
@@ -4869,13 +4872,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -4883,10 +4886,10 @@
         <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4894,37 +4897,37 @@
         <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C3" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B6">
         <v>2071234567</v>
@@ -4935,7 +4938,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B7">
         <v>7712345678</v>
@@ -4946,233 +4949,233 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C8" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C9" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B10" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C10" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B11" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C11" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B12" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C12" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B13" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C13" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C14" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B15" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C15" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B16" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C16" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B17" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C17" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B18" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C18" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B19" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C19" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B20" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C20" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B21" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C21" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B22" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C22" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B23" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C23" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B24" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C24" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B25" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C25" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B26" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C26" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B27" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C27" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B28" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C28" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: sync framework updates and report metadata
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/CarePlan/LSTP_CarePlan_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/CarePlan/LSTP_CarePlan_WF001.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrishnan6\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\CarePlan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B1FABB-377E-42EE-B8B7-5D8FE9A8B2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A59A6E79-C85E-49EF-A2ED-4B398540410E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{33E707BA-C33D-4108-BB34-C72B89CD78DB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="369">
   <si>
     <t>StepNo</t>
   </si>
@@ -78,9 +78,6 @@
   </si>
   <si>
     <t>launchUrl</t>
-  </si>
-  <si>
-    <t>http://dxcappchne8097a.cscidp.net/webclient_sso/extlogon.aspx?idp=oidnatlogon&amp;IsClientInfoNotRequired=true</t>
   </si>
   <si>
     <t>Login with valid credentials</t>
@@ -1605,25 +1602,22 @@
       <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="J2" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" t="s">
+      <c r="J3" t="s">
         <v>16</v>
-      </c>
-      <c r="J3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1631,13 +1625,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
+      <c r="F4" t="s">
         <v>19</v>
-      </c>
-      <c r="F4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1645,16 +1639,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
         <v>21</v>
       </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>22</v>
-      </c>
-      <c r="F5" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1662,13 +1656,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
         <v>19</v>
-      </c>
-      <c r="F6" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -1676,16 +1670,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>364</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
         <v>365</v>
       </c>
-      <c r="C7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" t="s">
-        <v>366</v>
-      </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1693,13 +1687,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" t="s">
         <v>25</v>
       </c>
-      <c r="F8" t="s">
+      <c r="J8" t="s">
         <v>26</v>
-      </c>
-      <c r="J8" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1707,19 +1701,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
         <v>28</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>29</v>
       </c>
-      <c r="D9" t="s">
+      <c r="F9" t="s">
         <v>30</v>
       </c>
-      <c r="F9" t="s">
+      <c r="J9" t="s">
         <v>31</v>
-      </c>
-      <c r="J9" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1727,16 +1721,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>366</v>
+      </c>
+      <c r="D10" t="s">
         <v>33</v>
       </c>
-      <c r="C10" t="s">
-        <v>367</v>
-      </c>
-      <c r="D10" t="s">
-        <v>34</v>
-      </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1744,13 +1738,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1758,16 +1752,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" t="s">
         <v>36</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>37</v>
       </c>
-      <c r="D12" t="s">
-        <v>38</v>
-      </c>
       <c r="F12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -1775,13 +1769,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
         <v>39</v>
       </c>
-      <c r="C13" t="s">
-        <v>40</v>
-      </c>
       <c r="F13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1789,19 +1783,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" t="s">
         <v>41</v>
       </c>
-      <c r="C14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="F14" t="s">
+        <v>30</v>
+      </c>
+      <c r="K14" t="s">
         <v>42</v>
-      </c>
-      <c r="F14" t="s">
-        <v>31</v>
-      </c>
-      <c r="K14" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1809,19 +1803,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" t="s">
         <v>30</v>
       </c>
-      <c r="F15" t="s">
+      <c r="J15" t="s">
         <v>31</v>
-      </c>
-      <c r="J15" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1829,19 +1823,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" t="s">
         <v>45</v>
       </c>
-      <c r="C16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="F16" t="s">
+        <v>30</v>
+      </c>
+      <c r="K16" t="s">
         <v>46</v>
-      </c>
-      <c r="F16" t="s">
-        <v>31</v>
-      </c>
-      <c r="K16" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1849,16 +1843,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -1866,13 +1860,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -1880,16 +1874,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -1897,22 +1891,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" t="s">
         <v>50</v>
       </c>
-      <c r="C20" t="s">
-        <v>40</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="F20" t="s">
+        <v>30</v>
+      </c>
+      <c r="J20" t="s">
+        <v>283</v>
+      </c>
+      <c r="K20" t="s">
         <v>51</v>
-      </c>
-      <c r="F20" t="s">
-        <v>31</v>
-      </c>
-      <c r="J20" t="s">
-        <v>284</v>
-      </c>
-      <c r="K20" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -1920,19 +1914,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" t="s">
         <v>53</v>
       </c>
-      <c r="C21" t="s">
-        <v>40</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="F21" t="s">
         <v>54</v>
       </c>
-      <c r="F21" t="s">
+      <c r="K21" t="s">
         <v>55</v>
-      </c>
-      <c r="K21" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -1940,19 +1934,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" t="s">
         <v>57</v>
       </c>
-      <c r="C22" t="s">
-        <v>40</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="F22" t="s">
+        <v>30</v>
+      </c>
+      <c r="K22" t="s">
         <v>58</v>
-      </c>
-      <c r="F22" t="s">
-        <v>31</v>
-      </c>
-      <c r="K22" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -1960,19 +1954,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" t="s">
         <v>60</v>
       </c>
-      <c r="C23" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="F23" t="s">
+        <v>30</v>
+      </c>
+      <c r="K23" t="s">
         <v>61</v>
-      </c>
-      <c r="F23" t="s">
-        <v>31</v>
-      </c>
-      <c r="K23" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -1980,19 +1974,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" t="s">
         <v>63</v>
       </c>
-      <c r="C24" t="s">
-        <v>40</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="F24" t="s">
+        <v>30</v>
+      </c>
+      <c r="K24" t="s">
         <v>64</v>
-      </c>
-      <c r="F24" t="s">
-        <v>31</v>
-      </c>
-      <c r="K24" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -2000,16 +1994,16 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" t="s">
         <v>66</v>
       </c>
-      <c r="C25" t="s">
-        <v>40</v>
-      </c>
-      <c r="D25" t="s">
-        <v>67</v>
-      </c>
       <c r="F25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -2017,13 +2011,13 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -2031,19 +2025,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" t="s">
+        <v>39</v>
+      </c>
+      <c r="D27" t="s">
         <v>69</v>
       </c>
-      <c r="C27" t="s">
-        <v>40</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="F27" t="s">
+        <v>54</v>
+      </c>
+      <c r="K27" t="s">
         <v>70</v>
-      </c>
-      <c r="F27" t="s">
-        <v>55</v>
-      </c>
-      <c r="K27" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -2051,19 +2045,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
+        <v>71</v>
+      </c>
+      <c r="C28" t="s">
+        <v>39</v>
+      </c>
+      <c r="D28" t="s">
         <v>72</v>
       </c>
-      <c r="C28" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="F28" t="s">
+        <v>54</v>
+      </c>
+      <c r="K28" t="s">
         <v>73</v>
-      </c>
-      <c r="F28" t="s">
-        <v>55</v>
-      </c>
-      <c r="K28" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -2071,19 +2065,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" t="s">
         <v>75</v>
       </c>
-      <c r="C29" t="s">
-        <v>40</v>
-      </c>
-      <c r="D29" t="s">
+      <c r="F29" t="s">
+        <v>54</v>
+      </c>
+      <c r="K29" t="s">
         <v>76</v>
-      </c>
-      <c r="F29" t="s">
-        <v>55</v>
-      </c>
-      <c r="K29" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -2091,19 +2085,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
+        <v>77</v>
+      </c>
+      <c r="C30" t="s">
+        <v>39</v>
+      </c>
+      <c r="D30" t="s">
         <v>78</v>
       </c>
-      <c r="C30" t="s">
-        <v>40</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="F30" t="s">
+        <v>54</v>
+      </c>
+      <c r="K30" t="s">
         <v>79</v>
-      </c>
-      <c r="F30" t="s">
-        <v>55</v>
-      </c>
-      <c r="K30" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -2111,19 +2105,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
+        <v>80</v>
+      </c>
+      <c r="C31" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" t="s">
         <v>81</v>
       </c>
-      <c r="C31" t="s">
-        <v>40</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="F31" t="s">
+        <v>54</v>
+      </c>
+      <c r="K31" t="s">
         <v>82</v>
-      </c>
-      <c r="F31" t="s">
-        <v>55</v>
-      </c>
-      <c r="K31" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -2131,19 +2125,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
+        <v>83</v>
+      </c>
+      <c r="C32" t="s">
+        <v>39</v>
+      </c>
+      <c r="D32" t="s">
         <v>84</v>
       </c>
-      <c r="C32" t="s">
-        <v>40</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="F32" t="s">
+        <v>54</v>
+      </c>
+      <c r="K32" t="s">
         <v>85</v>
-      </c>
-      <c r="F32" t="s">
-        <v>55</v>
-      </c>
-      <c r="K32" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -2151,16 +2145,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" t="s">
+        <v>39</v>
+      </c>
+      <c r="D33" t="s">
         <v>87</v>
       </c>
-      <c r="C33" t="s">
-        <v>40</v>
-      </c>
-      <c r="D33" t="s">
-        <v>88</v>
-      </c>
       <c r="F33" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -2168,13 +2162,13 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
+        <v>88</v>
+      </c>
+      <c r="C34" t="s">
         <v>89</v>
       </c>
-      <c r="C34" t="s">
-        <v>90</v>
-      </c>
       <c r="F34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -2182,19 +2176,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
+        <v>90</v>
+      </c>
+      <c r="C35" t="s">
+        <v>89</v>
+      </c>
+      <c r="D35" t="s">
         <v>91</v>
       </c>
-      <c r="C35" t="s">
-        <v>90</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="F35" t="s">
         <v>92</v>
       </c>
-      <c r="F35" t="s">
+      <c r="J35" t="s">
         <v>93</v>
-      </c>
-      <c r="J35" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -2202,22 +2196,22 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
+        <v>94</v>
+      </c>
+      <c r="C36" t="s">
+        <v>89</v>
+      </c>
+      <c r="D36" t="s">
+        <v>91</v>
+      </c>
+      <c r="F36" t="s">
         <v>95</v>
       </c>
-      <c r="C36" t="s">
-        <v>90</v>
-      </c>
-      <c r="D36" t="s">
-        <v>92</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
         <v>96</v>
       </c>
-      <c r="G36" t="s">
+      <c r="H36" t="s">
         <v>97</v>
-      </c>
-      <c r="H36" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -2225,16 +2219,16 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37" t="s">
+        <v>89</v>
+      </c>
+      <c r="D37" t="s">
         <v>99</v>
       </c>
-      <c r="C37" t="s">
-        <v>90</v>
-      </c>
-      <c r="D37" t="s">
-        <v>100</v>
-      </c>
       <c r="F37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
@@ -2242,13 +2236,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C38" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" t="s">
         <v>19</v>
-      </c>
-      <c r="F38" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
@@ -2256,16 +2250,16 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" t="s">
         <v>102</v>
       </c>
-      <c r="C39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D39" t="s">
-        <v>103</v>
-      </c>
       <c r="F39" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
@@ -2273,13 +2267,13 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F40" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
@@ -2287,19 +2281,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C41" t="s">
+        <v>28</v>
+      </c>
+      <c r="D41" t="s">
         <v>29</v>
       </c>
-      <c r="D41" t="s">
+      <c r="F41" t="s">
         <v>30</v>
       </c>
-      <c r="F41" t="s">
+      <c r="J41" t="s">
         <v>31</v>
-      </c>
-      <c r="J41" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
@@ -2307,16 +2301,16 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" t="s">
+        <v>28</v>
+      </c>
+      <c r="D42" t="s">
         <v>33</v>
       </c>
-      <c r="C42" t="s">
-        <v>29</v>
-      </c>
-      <c r="D42" t="s">
-        <v>34</v>
-      </c>
       <c r="F42" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -2324,13 +2318,13 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C43" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F43" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -2338,16 +2332,16 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>105</v>
+      </c>
+      <c r="C44" t="s">
         <v>106</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>107</v>
       </c>
-      <c r="D44" t="s">
-        <v>108</v>
-      </c>
       <c r="F44" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -2355,13 +2349,13 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
+        <v>108</v>
+      </c>
+      <c r="C45" t="s">
         <v>109</v>
       </c>
-      <c r="C45" t="s">
-        <v>110</v>
-      </c>
       <c r="F45" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
@@ -2369,22 +2363,22 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
+        <v>110</v>
+      </c>
+      <c r="C46" t="s">
+        <v>109</v>
+      </c>
+      <c r="D46" t="s">
         <v>111</v>
       </c>
-      <c r="C46" t="s">
-        <v>110</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="F46" t="s">
+        <v>95</v>
+      </c>
+      <c r="G46" t="s">
         <v>112</v>
       </c>
-      <c r="F46" t="s">
-        <v>96</v>
-      </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>113</v>
-      </c>
-      <c r="H46" t="s">
-        <v>114</v>
       </c>
       <c r="J46" t="b">
         <v>1</v>
@@ -2395,19 +2389,19 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
+        <v>114</v>
+      </c>
+      <c r="C47" t="s">
+        <v>109</v>
+      </c>
+      <c r="D47" t="s">
+        <v>111</v>
+      </c>
+      <c r="F47" t="s">
+        <v>92</v>
+      </c>
+      <c r="J47" t="s">
         <v>115</v>
-      </c>
-      <c r="C47" t="s">
-        <v>110</v>
-      </c>
-      <c r="D47" t="s">
-        <v>112</v>
-      </c>
-      <c r="F47" t="s">
-        <v>93</v>
-      </c>
-      <c r="J47" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
@@ -2415,16 +2409,16 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
+        <v>116</v>
+      </c>
+      <c r="C48" t="s">
+        <v>109</v>
+      </c>
+      <c r="D48" t="s">
         <v>117</v>
       </c>
-      <c r="C48" t="s">
-        <v>110</v>
-      </c>
-      <c r="D48" t="s">
-        <v>118</v>
-      </c>
       <c r="F48" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -2432,13 +2426,13 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C49" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F49" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -2446,16 +2440,16 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
+        <v>119</v>
+      </c>
+      <c r="C50" t="s">
+        <v>109</v>
+      </c>
+      <c r="D50" t="s">
         <v>120</v>
       </c>
-      <c r="C50" t="s">
-        <v>110</v>
-      </c>
-      <c r="D50" t="s">
-        <v>121</v>
-      </c>
       <c r="F50" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -2463,13 +2457,13 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
+        <v>121</v>
+      </c>
+      <c r="C51" t="s">
         <v>122</v>
       </c>
-      <c r="C51" t="s">
-        <v>123</v>
-      </c>
       <c r="F51" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
@@ -2477,19 +2471,19 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
+        <v>123</v>
+      </c>
+      <c r="C52" t="s">
+        <v>122</v>
+      </c>
+      <c r="D52" t="s">
         <v>124</v>
       </c>
-      <c r="C52" t="s">
-        <v>123</v>
-      </c>
-      <c r="D52" t="s">
+      <c r="F52" t="s">
+        <v>54</v>
+      </c>
+      <c r="K52" t="s">
         <v>125</v>
-      </c>
-      <c r="F52" t="s">
-        <v>55</v>
-      </c>
-      <c r="K52" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
@@ -2497,19 +2491,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
+        <v>126</v>
+      </c>
+      <c r="C53" t="s">
+        <v>122</v>
+      </c>
+      <c r="D53" t="s">
         <v>127</v>
       </c>
-      <c r="C53" t="s">
-        <v>123</v>
-      </c>
-      <c r="D53" t="s">
+      <c r="F53" t="s">
+        <v>54</v>
+      </c>
+      <c r="K53" t="s">
         <v>128</v>
-      </c>
-      <c r="F53" t="s">
-        <v>55</v>
-      </c>
-      <c r="K53" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -2517,19 +2511,19 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
+        <v>129</v>
+      </c>
+      <c r="C54" t="s">
+        <v>122</v>
+      </c>
+      <c r="D54" t="s">
         <v>130</v>
       </c>
-      <c r="C54" t="s">
-        <v>123</v>
-      </c>
-      <c r="D54" t="s">
+      <c r="F54" t="s">
+        <v>54</v>
+      </c>
+      <c r="K54" t="s">
         <v>131</v>
-      </c>
-      <c r="F54" t="s">
-        <v>55</v>
-      </c>
-      <c r="K54" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
@@ -2537,19 +2531,19 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
+        <v>132</v>
+      </c>
+      <c r="C55" t="s">
+        <v>122</v>
+      </c>
+      <c r="D55" t="s">
         <v>133</v>
       </c>
-      <c r="C55" t="s">
-        <v>123</v>
-      </c>
-      <c r="D55" t="s">
+      <c r="F55" t="s">
+        <v>54</v>
+      </c>
+      <c r="K55" t="s">
         <v>134</v>
-      </c>
-      <c r="F55" t="s">
-        <v>55</v>
-      </c>
-      <c r="K55" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -2557,16 +2551,16 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
+        <v>135</v>
+      </c>
+      <c r="C56" t="s">
+        <v>122</v>
+      </c>
+      <c r="D56" t="s">
         <v>136</v>
       </c>
-      <c r="C56" t="s">
-        <v>123</v>
-      </c>
-      <c r="D56" t="s">
-        <v>137</v>
-      </c>
       <c r="F56" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
@@ -2574,13 +2568,13 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C57" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F57" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
@@ -2588,22 +2582,22 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
+        <v>138</v>
+      </c>
+      <c r="C58" t="s">
         <v>139</v>
       </c>
-      <c r="C58" t="s">
-        <v>140</v>
-      </c>
       <c r="D58" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F58" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G58" t="s">
+        <v>112</v>
+      </c>
+      <c r="H58" t="s">
         <v>113</v>
-      </c>
-      <c r="H58" t="s">
-        <v>114</v>
       </c>
       <c r="J58" t="b">
         <v>1</v>
@@ -2614,10 +2608,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
+        <v>140</v>
+      </c>
+      <c r="F59" t="s">
         <v>141</v>
-      </c>
-      <c r="F59" t="s">
-        <v>142</v>
       </c>
       <c r="J59">
         <v>1</v>
@@ -2628,16 +2622,16 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C60" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D60" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F60" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -2645,16 +2639,16 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
+        <v>143</v>
+      </c>
+      <c r="C61" t="s">
+        <v>139</v>
+      </c>
+      <c r="D61" t="s">
         <v>144</v>
       </c>
-      <c r="C61" t="s">
-        <v>140</v>
-      </c>
-      <c r="D61" t="s">
-        <v>145</v>
-      </c>
       <c r="F61" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
@@ -2662,13 +2656,13 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
+        <v>145</v>
+      </c>
+      <c r="C62" t="s">
         <v>146</v>
       </c>
-      <c r="C62" t="s">
-        <v>147</v>
-      </c>
       <c r="F62" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
@@ -2676,19 +2670,19 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
+        <v>147</v>
+      </c>
+      <c r="C63" t="s">
+        <v>146</v>
+      </c>
+      <c r="D63" t="s">
         <v>148</v>
       </c>
-      <c r="C63" t="s">
-        <v>147</v>
-      </c>
-      <c r="D63" t="s">
+      <c r="F63" t="s">
+        <v>54</v>
+      </c>
+      <c r="K63" t="s">
         <v>149</v>
-      </c>
-      <c r="F63" t="s">
-        <v>55</v>
-      </c>
-      <c r="K63" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
@@ -2696,19 +2690,19 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
+        <v>150</v>
+      </c>
+      <c r="C64" t="s">
+        <v>146</v>
+      </c>
+      <c r="D64" t="s">
         <v>151</v>
       </c>
-      <c r="C64" t="s">
-        <v>147</v>
-      </c>
-      <c r="D64" t="s">
+      <c r="F64" t="s">
+        <v>54</v>
+      </c>
+      <c r="K64" t="s">
         <v>152</v>
-      </c>
-      <c r="F64" t="s">
-        <v>55</v>
-      </c>
-      <c r="K64" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
@@ -2716,19 +2710,19 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
+        <v>153</v>
+      </c>
+      <c r="C65" t="s">
+        <v>146</v>
+      </c>
+      <c r="D65" t="s">
         <v>154</v>
       </c>
-      <c r="C65" t="s">
-        <v>147</v>
-      </c>
-      <c r="D65" t="s">
+      <c r="F65" t="s">
+        <v>54</v>
+      </c>
+      <c r="K65" t="s">
         <v>155</v>
-      </c>
-      <c r="F65" t="s">
-        <v>55</v>
-      </c>
-      <c r="K65" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
@@ -2736,19 +2730,19 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
+        <v>156</v>
+      </c>
+      <c r="C66" t="s">
+        <v>146</v>
+      </c>
+      <c r="D66" t="s">
         <v>157</v>
       </c>
-      <c r="C66" t="s">
-        <v>147</v>
-      </c>
-      <c r="D66" t="s">
+      <c r="F66" t="s">
+        <v>54</v>
+      </c>
+      <c r="K66" t="s">
         <v>158</v>
-      </c>
-      <c r="F66" t="s">
-        <v>55</v>
-      </c>
-      <c r="K66" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -2756,16 +2750,16 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C67" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D67" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F67" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -2773,13 +2767,13 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
+        <v>160</v>
+      </c>
+      <c r="C68" t="s">
         <v>161</v>
       </c>
-      <c r="C68" t="s">
-        <v>162</v>
-      </c>
       <c r="F68" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
@@ -2787,16 +2781,16 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C69" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D69" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F69" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
@@ -2804,13 +2798,13 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C70" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F70" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -2818,22 +2812,22 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C71" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D71" t="s">
+        <v>111</v>
+      </c>
+      <c r="F71" t="s">
+        <v>95</v>
+      </c>
+      <c r="G71" t="s">
         <v>112</v>
       </c>
-      <c r="F71" t="s">
-        <v>96</v>
-      </c>
-      <c r="G71" t="s">
+      <c r="H71" t="s">
         <v>113</v>
-      </c>
-      <c r="H71" t="s">
-        <v>114</v>
       </c>
       <c r="J71" t="b">
         <v>1</v>
@@ -2844,10 +2838,10 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F72" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J72">
         <v>1</v>
@@ -2858,16 +2852,16 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
+        <v>166</v>
+      </c>
+      <c r="C73" t="s">
+        <v>109</v>
+      </c>
+      <c r="D73" t="s">
         <v>167</v>
       </c>
-      <c r="C73" t="s">
-        <v>110</v>
-      </c>
-      <c r="D73" t="s">
-        <v>168</v>
-      </c>
       <c r="F73" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -2875,13 +2869,13 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C74" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F74" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -2889,22 +2883,22 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C75" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D75" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F75" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G75" t="s">
+        <v>112</v>
+      </c>
+      <c r="H75" t="s">
         <v>113</v>
-      </c>
-      <c r="H75" t="s">
-        <v>114</v>
       </c>
       <c r="J75" t="b">
         <v>1</v>
@@ -2915,10 +2909,10 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F76" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J76">
         <v>1</v>
@@ -2929,16 +2923,16 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
+        <v>171</v>
+      </c>
+      <c r="C77" t="s">
+        <v>139</v>
+      </c>
+      <c r="D77" t="s">
         <v>172</v>
       </c>
-      <c r="C77" t="s">
-        <v>140</v>
-      </c>
-      <c r="D77" t="s">
-        <v>173</v>
-      </c>
       <c r="F77" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
@@ -2946,13 +2940,13 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
+        <v>173</v>
+      </c>
+      <c r="C78" t="s">
         <v>174</v>
       </c>
-      <c r="C78" t="s">
-        <v>175</v>
-      </c>
       <c r="F78" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
@@ -2960,19 +2954,19 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
+        <v>175</v>
+      </c>
+      <c r="C79" t="s">
+        <v>174</v>
+      </c>
+      <c r="D79" t="s">
         <v>176</v>
       </c>
-      <c r="C79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D79" t="s">
+      <c r="F79" t="s">
+        <v>30</v>
+      </c>
+      <c r="K79" t="s">
         <v>177</v>
-      </c>
-      <c r="F79" t="s">
-        <v>31</v>
-      </c>
-      <c r="K79" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -2980,16 +2974,16 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C80" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D80" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F80" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -2997,13 +2991,13 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C81" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F81" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
@@ -3011,16 +3005,16 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
+        <v>180</v>
+      </c>
+      <c r="C82" t="s">
         <v>181</v>
       </c>
-      <c r="C82" t="s">
-        <v>182</v>
-      </c>
       <c r="D82" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F82" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -3028,13 +3022,13 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C83" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F83" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
@@ -3042,16 +3036,16 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
+        <v>183</v>
+      </c>
+      <c r="C84" t="s">
+        <v>181</v>
+      </c>
+      <c r="D84" t="s">
         <v>184</v>
       </c>
-      <c r="C84" t="s">
-        <v>182</v>
-      </c>
-      <c r="D84" t="s">
-        <v>185</v>
-      </c>
       <c r="F84" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
@@ -3059,13 +3053,13 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
+        <v>185</v>
+      </c>
+      <c r="C85" t="s">
         <v>186</v>
       </c>
-      <c r="C85" t="s">
-        <v>187</v>
-      </c>
       <c r="F85" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
@@ -3073,16 +3067,16 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
+        <v>187</v>
+      </c>
+      <c r="C86" t="s">
+        <v>186</v>
+      </c>
+      <c r="D86" t="s">
         <v>188</v>
       </c>
-      <c r="C86" t="s">
-        <v>187</v>
-      </c>
-      <c r="D86" t="s">
-        <v>189</v>
-      </c>
       <c r="F86" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
@@ -3090,16 +3084,16 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
+        <v>189</v>
+      </c>
+      <c r="C87" t="s">
+        <v>186</v>
+      </c>
+      <c r="D87" t="s">
         <v>190</v>
       </c>
-      <c r="C87" t="s">
-        <v>187</v>
-      </c>
-      <c r="D87" t="s">
-        <v>191</v>
-      </c>
       <c r="F87" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
@@ -3107,13 +3101,13 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C88" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F88" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
@@ -3121,10 +3115,10 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F89" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J89">
         <v>1</v>
@@ -3135,22 +3129,22 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C90" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D90" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F90" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G90" t="s">
+        <v>112</v>
+      </c>
+      <c r="H90" t="s">
         <v>113</v>
-      </c>
-      <c r="H90" t="s">
-        <v>114</v>
       </c>
       <c r="J90" t="b">
         <v>1</v>
@@ -3161,22 +3155,22 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C91" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D91" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F91" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G91" t="s">
+        <v>112</v>
+      </c>
+      <c r="H91" t="s">
         <v>113</v>
-      </c>
-      <c r="H91" t="s">
-        <v>114</v>
       </c>
       <c r="J91" t="b">
         <v>1</v>
@@ -3187,10 +3181,10 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F92" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J92">
         <v>1</v>
@@ -3201,16 +3195,16 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D93" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F93" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
@@ -3218,16 +3212,16 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
+        <v>197</v>
+      </c>
+      <c r="C94" t="s">
+        <v>139</v>
+      </c>
+      <c r="D94" t="s">
         <v>198</v>
       </c>
-      <c r="C94" t="s">
-        <v>140</v>
-      </c>
-      <c r="D94" t="s">
-        <v>199</v>
-      </c>
       <c r="F94" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.25">
@@ -3235,13 +3229,13 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
+        <v>199</v>
+      </c>
+      <c r="C95" t="s">
         <v>200</v>
       </c>
-      <c r="C95" t="s">
-        <v>201</v>
-      </c>
       <c r="F95" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
@@ -3249,19 +3243,19 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
+        <v>201</v>
+      </c>
+      <c r="C96" t="s">
+        <v>200</v>
+      </c>
+      <c r="D96" t="s">
         <v>202</v>
       </c>
-      <c r="C96" t="s">
-        <v>201</v>
-      </c>
-      <c r="D96" t="s">
+      <c r="F96" t="s">
+        <v>54</v>
+      </c>
+      <c r="K96" t="s">
         <v>203</v>
-      </c>
-      <c r="F96" t="s">
-        <v>55</v>
-      </c>
-      <c r="K96" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.25">
@@ -3269,13 +3263,13 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
+        <v>204</v>
+      </c>
+      <c r="C97" t="s">
         <v>205</v>
       </c>
-      <c r="C97" t="s">
-        <v>206</v>
-      </c>
       <c r="F97" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
@@ -3283,16 +3277,16 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C98" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D98" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F98" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
@@ -3300,13 +3294,13 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
+        <v>185</v>
+      </c>
+      <c r="C99" t="s">
         <v>186</v>
       </c>
-      <c r="C99" t="s">
-        <v>187</v>
-      </c>
       <c r="F99" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
@@ -3314,16 +3308,16 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
+        <v>207</v>
+      </c>
+      <c r="C100" t="s">
+        <v>186</v>
+      </c>
+      <c r="D100" t="s">
         <v>208</v>
       </c>
-      <c r="C100" t="s">
-        <v>187</v>
-      </c>
-      <c r="D100" t="s">
-        <v>209</v>
-      </c>
       <c r="F100" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
@@ -3331,16 +3325,16 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C101" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D101" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F101" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
@@ -3348,13 +3342,13 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C102" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F102" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
@@ -3362,10 +3356,10 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F103" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J103">
         <v>1</v>
@@ -3376,22 +3370,22 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C104" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D104" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F104" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G104" t="s">
+        <v>112</v>
+      </c>
+      <c r="H104" t="s">
         <v>113</v>
-      </c>
-      <c r="H104" t="s">
-        <v>114</v>
       </c>
       <c r="J104" t="b">
         <v>1</v>
@@ -3402,22 +3396,22 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C105" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D105" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F105" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G105" t="s">
+        <v>112</v>
+      </c>
+      <c r="H105" t="s">
         <v>113</v>
-      </c>
-      <c r="H105" t="s">
-        <v>114</v>
       </c>
       <c r="J105" t="b">
         <v>1</v>
@@ -3428,10 +3422,10 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F106" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J106">
         <v>1</v>
@@ -3442,16 +3436,16 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C107" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D107" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F107" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
@@ -3459,16 +3453,16 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
+        <v>216</v>
+      </c>
+      <c r="C108" t="s">
+        <v>139</v>
+      </c>
+      <c r="D108" t="s">
         <v>217</v>
       </c>
-      <c r="C108" t="s">
-        <v>140</v>
-      </c>
-      <c r="D108" t="s">
-        <v>218</v>
-      </c>
       <c r="F108" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.25">
@@ -3476,13 +3470,13 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C109" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F109" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
@@ -3490,19 +3484,19 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
+        <v>219</v>
+      </c>
+      <c r="C110" t="s">
+        <v>200</v>
+      </c>
+      <c r="D110" t="s">
         <v>220</v>
       </c>
-      <c r="C110" t="s">
-        <v>201</v>
-      </c>
-      <c r="D110" t="s">
+      <c r="F110" t="s">
+        <v>30</v>
+      </c>
+      <c r="K110" t="s">
         <v>221</v>
-      </c>
-      <c r="F110" t="s">
-        <v>31</v>
-      </c>
-      <c r="K110" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.25">
@@ -3510,13 +3504,13 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
+        <v>222</v>
+      </c>
+      <c r="C111" t="s">
         <v>223</v>
       </c>
-      <c r="C111" t="s">
-        <v>224</v>
-      </c>
       <c r="F111" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.25">
@@ -3524,16 +3518,16 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C112" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D112" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F112" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.25">
@@ -3541,13 +3535,13 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
+        <v>185</v>
+      </c>
+      <c r="C113" t="s">
         <v>186</v>
       </c>
-      <c r="C113" t="s">
-        <v>187</v>
-      </c>
       <c r="F113" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.25">
@@ -3555,16 +3549,16 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C114" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D114" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F114" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
@@ -3572,13 +3566,13 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C115" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F115" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
@@ -3586,10 +3580,10 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F116" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J116">
         <v>1</v>
@@ -3600,22 +3594,22 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C117" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D117" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F117" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G117" t="s">
+        <v>112</v>
+      </c>
+      <c r="H117" t="s">
         <v>113</v>
-      </c>
-      <c r="H117" t="s">
-        <v>114</v>
       </c>
       <c r="J117" t="b">
         <v>1</v>
@@ -3626,22 +3620,22 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C118" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D118" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F118" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G118" t="s">
+        <v>112</v>
+      </c>
+      <c r="H118" t="s">
         <v>113</v>
-      </c>
-      <c r="H118" t="s">
-        <v>114</v>
       </c>
       <c r="J118" t="b">
         <v>1</v>
@@ -3652,10 +3646,10 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F119" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J119">
         <v>1</v>
@@ -3666,16 +3660,16 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C120" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D120" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F120" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
@@ -3683,16 +3677,16 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
+        <v>232</v>
+      </c>
+      <c r="C121" t="s">
+        <v>139</v>
+      </c>
+      <c r="D121" t="s">
         <v>233</v>
       </c>
-      <c r="C121" t="s">
-        <v>140</v>
-      </c>
-      <c r="D121" t="s">
-        <v>234</v>
-      </c>
       <c r="F121" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
@@ -3700,13 +3694,13 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
+        <v>234</v>
+      </c>
+      <c r="C122" t="s">
         <v>235</v>
       </c>
-      <c r="C122" t="s">
-        <v>236</v>
-      </c>
       <c r="F122" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
@@ -3714,19 +3708,19 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
+        <v>236</v>
+      </c>
+      <c r="C123" t="s">
+        <v>235</v>
+      </c>
+      <c r="D123" t="s">
         <v>237</v>
       </c>
-      <c r="C123" t="s">
-        <v>236</v>
-      </c>
-      <c r="D123" t="s">
+      <c r="F123" t="s">
+        <v>54</v>
+      </c>
+      <c r="K123" t="s">
         <v>238</v>
-      </c>
-      <c r="F123" t="s">
-        <v>55</v>
-      </c>
-      <c r="K123" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
@@ -3734,13 +3728,13 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
+        <v>239</v>
+      </c>
+      <c r="C124" t="s">
         <v>240</v>
       </c>
-      <c r="C124" t="s">
-        <v>241</v>
-      </c>
       <c r="F124" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
@@ -3748,16 +3742,16 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
+        <v>241</v>
+      </c>
+      <c r="C125" t="s">
+        <v>240</v>
+      </c>
+      <c r="D125" t="s">
         <v>242</v>
       </c>
-      <c r="C125" t="s">
-        <v>241</v>
-      </c>
-      <c r="D125" t="s">
-        <v>243</v>
-      </c>
       <c r="F125" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
@@ -3765,13 +3759,13 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C126" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F126" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
@@ -3779,10 +3773,10 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F127" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J127">
         <v>1</v>
@@ -3793,22 +3787,22 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C128" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D128" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F128" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G128" t="s">
+        <v>112</v>
+      </c>
+      <c r="H128" t="s">
         <v>113</v>
-      </c>
-      <c r="H128" t="s">
-        <v>114</v>
       </c>
       <c r="J128" t="b">
         <v>1</v>
@@ -3819,22 +3813,22 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C129" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D129" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F129" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G129" t="s">
+        <v>112</v>
+      </c>
+      <c r="H129" t="s">
         <v>113</v>
-      </c>
-      <c r="H129" t="s">
-        <v>114</v>
       </c>
       <c r="J129" t="b">
         <v>1</v>
@@ -3845,10 +3839,10 @@
         <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F130" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J130">
         <v>1</v>
@@ -3859,16 +3853,16 @@
         <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C131" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D131" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F131" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.25">
@@ -3876,16 +3870,16 @@
         <v>131</v>
       </c>
       <c r="B132" t="s">
+        <v>232</v>
+      </c>
+      <c r="C132" t="s">
+        <v>139</v>
+      </c>
+      <c r="D132" t="s">
         <v>233</v>
       </c>
-      <c r="C132" t="s">
-        <v>140</v>
-      </c>
-      <c r="D132" t="s">
-        <v>234</v>
-      </c>
       <c r="F132" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="133" spans="1:11" x14ac:dyDescent="0.25">
@@ -3893,13 +3887,13 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
+        <v>234</v>
+      </c>
+      <c r="C133" t="s">
         <v>235</v>
       </c>
-      <c r="C133" t="s">
-        <v>236</v>
-      </c>
       <c r="F133" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.25">
@@ -3907,19 +3901,19 @@
         <v>133</v>
       </c>
       <c r="B134" t="s">
+        <v>249</v>
+      </c>
+      <c r="C134" t="s">
+        <v>235</v>
+      </c>
+      <c r="D134" t="s">
         <v>250</v>
       </c>
-      <c r="C134" t="s">
-        <v>236</v>
-      </c>
-      <c r="D134" t="s">
+      <c r="F134" t="s">
+        <v>54</v>
+      </c>
+      <c r="K134" t="s">
         <v>251</v>
-      </c>
-      <c r="F134" t="s">
-        <v>55</v>
-      </c>
-      <c r="K134" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.25">
@@ -3927,13 +3921,13 @@
         <v>134</v>
       </c>
       <c r="B135" t="s">
+        <v>239</v>
+      </c>
+      <c r="C135" t="s">
         <v>240</v>
       </c>
-      <c r="C135" t="s">
-        <v>241</v>
-      </c>
       <c r="F135" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="136" spans="1:11" x14ac:dyDescent="0.25">
@@ -3941,16 +3935,16 @@
         <v>135</v>
       </c>
       <c r="B136" t="s">
+        <v>252</v>
+      </c>
+      <c r="C136" t="s">
+        <v>240</v>
+      </c>
+      <c r="D136" t="s">
         <v>253</v>
       </c>
-      <c r="C136" t="s">
-        <v>241</v>
-      </c>
-      <c r="D136" t="s">
-        <v>254</v>
-      </c>
       <c r="F136" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="137" spans="1:11" x14ac:dyDescent="0.25">
@@ -3958,13 +3952,13 @@
         <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C137" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F137" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="138" spans="1:11" x14ac:dyDescent="0.25">
@@ -3972,10 +3966,10 @@
         <v>137</v>
       </c>
       <c r="B138" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F138" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J138">
         <v>1</v>
@@ -3986,22 +3980,22 @@
         <v>138</v>
       </c>
       <c r="B139" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C139" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D139" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F139" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G139" t="s">
+        <v>112</v>
+      </c>
+      <c r="H139" t="s">
         <v>113</v>
-      </c>
-      <c r="H139" t="s">
-        <v>114</v>
       </c>
       <c r="J139" t="b">
         <v>1</v>
@@ -4012,22 +4006,22 @@
         <v>139</v>
       </c>
       <c r="B140" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C140" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D140" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F140" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G140" t="s">
+        <v>112</v>
+      </c>
+      <c r="H140" t="s">
         <v>113</v>
-      </c>
-      <c r="H140" t="s">
-        <v>114</v>
       </c>
       <c r="J140" t="b">
         <v>1</v>
@@ -4038,10 +4032,10 @@
         <v>140</v>
       </c>
       <c r="B141" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F141" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J141">
         <v>1</v>
@@ -4052,16 +4046,16 @@
         <v>141</v>
       </c>
       <c r="B142" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C142" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D142" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F142" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="143" spans="1:11" x14ac:dyDescent="0.25">
@@ -4069,16 +4063,16 @@
         <v>142</v>
       </c>
       <c r="B143" t="s">
+        <v>232</v>
+      </c>
+      <c r="C143" t="s">
+        <v>139</v>
+      </c>
+      <c r="D143" t="s">
         <v>233</v>
       </c>
-      <c r="C143" t="s">
-        <v>140</v>
-      </c>
-      <c r="D143" t="s">
-        <v>234</v>
-      </c>
       <c r="F143" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.25">
@@ -4086,13 +4080,13 @@
         <v>143</v>
       </c>
       <c r="B144" t="s">
+        <v>234</v>
+      </c>
+      <c r="C144" t="s">
         <v>235</v>
       </c>
-      <c r="C144" t="s">
-        <v>236</v>
-      </c>
       <c r="F144" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="145" spans="1:11" x14ac:dyDescent="0.25">
@@ -4100,19 +4094,19 @@
         <v>144</v>
       </c>
       <c r="B145" t="s">
+        <v>260</v>
+      </c>
+      <c r="C145" t="s">
+        <v>235</v>
+      </c>
+      <c r="D145" t="s">
         <v>261</v>
       </c>
-      <c r="C145" t="s">
-        <v>236</v>
-      </c>
-      <c r="D145" t="s">
+      <c r="F145" t="s">
+        <v>54</v>
+      </c>
+      <c r="K145" t="s">
         <v>262</v>
-      </c>
-      <c r="F145" t="s">
-        <v>55</v>
-      </c>
-      <c r="K145" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="146" spans="1:11" x14ac:dyDescent="0.25">
@@ -4120,13 +4114,13 @@
         <v>145</v>
       </c>
       <c r="B146" t="s">
+        <v>239</v>
+      </c>
+      <c r="C146" t="s">
         <v>240</v>
       </c>
-      <c r="C146" t="s">
-        <v>241</v>
-      </c>
       <c r="F146" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="147" spans="1:11" x14ac:dyDescent="0.25">
@@ -4134,16 +4128,16 @@
         <v>146</v>
       </c>
       <c r="B147" t="s">
+        <v>263</v>
+      </c>
+      <c r="C147" t="s">
+        <v>240</v>
+      </c>
+      <c r="D147" t="s">
         <v>264</v>
       </c>
-      <c r="C147" t="s">
-        <v>241</v>
-      </c>
-      <c r="D147" t="s">
-        <v>265</v>
-      </c>
       <c r="F147" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="148" spans="1:11" x14ac:dyDescent="0.25">
@@ -4151,13 +4145,13 @@
         <v>147</v>
       </c>
       <c r="B148" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C148" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F148" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.25">
@@ -4165,10 +4159,10 @@
         <v>148</v>
       </c>
       <c r="B149" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F149" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J149">
         <v>1</v>
@@ -4179,22 +4173,22 @@
         <v>149</v>
       </c>
       <c r="B150" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C150" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D150" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F150" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G150" t="s">
+        <v>112</v>
+      </c>
+      <c r="H150" t="s">
         <v>113</v>
-      </c>
-      <c r="H150" t="s">
-        <v>114</v>
       </c>
       <c r="J150" t="b">
         <v>1</v>
@@ -4205,22 +4199,22 @@
         <v>150</v>
       </c>
       <c r="B151" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C151" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D151" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F151" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G151" t="s">
+        <v>112</v>
+      </c>
+      <c r="H151" t="s">
         <v>113</v>
-      </c>
-      <c r="H151" t="s">
-        <v>114</v>
       </c>
       <c r="J151" t="b">
         <v>1</v>
@@ -4231,16 +4225,16 @@
         <v>151</v>
       </c>
       <c r="B152" t="s">
+        <v>269</v>
+      </c>
+      <c r="C152" t="s">
+        <v>18</v>
+      </c>
+      <c r="D152" t="s">
         <v>270</v>
       </c>
-      <c r="C152" t="s">
-        <v>19</v>
-      </c>
-      <c r="D152" t="s">
-        <v>271</v>
-      </c>
       <c r="F152" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.25">
@@ -4248,16 +4242,16 @@
         <v>152</v>
       </c>
       <c r="B153" t="s">
+        <v>271</v>
+      </c>
+      <c r="C153" t="s">
+        <v>18</v>
+      </c>
+      <c r="D153" t="s">
         <v>272</v>
       </c>
-      <c r="C153" t="s">
-        <v>19</v>
-      </c>
-      <c r="D153" t="s">
-        <v>273</v>
-      </c>
       <c r="F153" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.25">
@@ -4265,10 +4259,10 @@
         <v>153</v>
       </c>
       <c r="B154" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F154" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J154">
         <v>3</v>
@@ -4292,394 +4286,394 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>277</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C2" t="s">
         <v>279</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>280</v>
-      </c>
-      <c r="D2" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C3" t="s">
+        <v>281</v>
+      </c>
+      <c r="D3" t="s">
         <v>282</v>
-      </c>
-      <c r="D3" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C4" t="s">
+        <v>283</v>
+      </c>
+      <c r="D4" t="s">
         <v>284</v>
-      </c>
-      <c r="D4" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C5" t="s">
+        <v>285</v>
+      </c>
+      <c r="D5" t="s">
         <v>286</v>
-      </c>
-      <c r="D5" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C6">
         <v>2071234567</v>
       </c>
       <c r="D6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C7">
         <v>7712345678</v>
       </c>
       <c r="D7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C8" t="s">
+        <v>289</v>
+      </c>
+      <c r="D8" t="s">
         <v>290</v>
-      </c>
-      <c r="D8" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C9" t="s">
+        <v>291</v>
+      </c>
+      <c r="D9" t="s">
         <v>292</v>
-      </c>
-      <c r="D9" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C10" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D10" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C11" t="s">
+        <v>294</v>
+      </c>
+      <c r="D11" t="s">
         <v>295</v>
-      </c>
-      <c r="D11" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C12" t="s">
+        <v>296</v>
+      </c>
+      <c r="D12" t="s">
         <v>297</v>
-      </c>
-      <c r="D12" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B13" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C13" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D13" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C14" t="s">
+        <v>299</v>
+      </c>
+      <c r="D14" t="s">
         <v>300</v>
-      </c>
-      <c r="D14" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B15" t="s">
+        <v>301</v>
+      </c>
+      <c r="C15" t="s">
         <v>302</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>303</v>
-      </c>
-      <c r="D15" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C16" t="s">
+        <v>304</v>
+      </c>
+      <c r="D16" t="s">
         <v>305</v>
-      </c>
-      <c r="D16" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C17" t="s">
+        <v>306</v>
+      </c>
+      <c r="D17" t="s">
         <v>307</v>
-      </c>
-      <c r="D17" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C18" t="s">
+        <v>308</v>
+      </c>
+      <c r="D18" t="s">
         <v>309</v>
-      </c>
-      <c r="D18" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B19" t="s">
+        <v>310</v>
+      </c>
+      <c r="C19" t="s">
         <v>311</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>312</v>
-      </c>
-      <c r="D19" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B20" t="s">
+        <v>310</v>
+      </c>
+      <c r="C20" t="s">
         <v>311</v>
       </c>
-      <c r="C20" t="s">
-        <v>312</v>
-      </c>
       <c r="D20" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B21" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C21" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D21" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B22" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C22" t="s">
+        <v>315</v>
+      </c>
+      <c r="D22" t="s">
         <v>316</v>
-      </c>
-      <c r="D22" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B23" t="s">
+        <v>317</v>
+      </c>
+      <c r="C23" t="s">
         <v>318</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>319</v>
-      </c>
-      <c r="D23" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B24" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C24" t="s">
+        <v>320</v>
+      </c>
+      <c r="D24" t="s">
         <v>321</v>
-      </c>
-      <c r="D24" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B25" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C25" t="s">
+        <v>322</v>
+      </c>
+      <c r="D25" t="s">
         <v>323</v>
-      </c>
-      <c r="D25" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B26" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C26" t="s">
+        <v>324</v>
+      </c>
+      <c r="D26" t="s">
         <v>325</v>
-      </c>
-      <c r="D26" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B27" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C27" t="s">
+        <v>326</v>
+      </c>
+      <c r="D27" t="s">
         <v>327</v>
-      </c>
-      <c r="D27" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B28" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C28" t="s">
+        <v>328</v>
+      </c>
+      <c r="D28" t="s">
         <v>329</v>
-      </c>
-      <c r="D28" t="s">
-        <v>330</v>
       </c>
     </row>
   </sheetData>
@@ -4698,71 +4692,71 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>331</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>333</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>335</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>338</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>340</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>342</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B9" s="2">
         <v>152</v>
@@ -4770,7 +4764,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B10" s="2">
         <v>20</v>
@@ -4778,7 +4772,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B11" s="2">
         <v>57</v>
@@ -4786,15 +4780,15 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>347</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B13" s="3">
         <v>46146</v>
@@ -4802,7 +4796,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B14" s="3">
         <v>46146</v>
@@ -4810,31 +4804,31 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>351</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>353</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>355</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B18" s="2">
         <v>17</v>
@@ -4842,18 +4836,18 @@
     </row>
     <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>358</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>360</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>361</v>
       </c>
     </row>
   </sheetData>
@@ -4872,62 +4866,62 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>362</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6">
         <v>2071234567</v>
@@ -4938,7 +4932,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B7">
         <v>7712345678</v>
@@ -4949,233 +4943,233 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C10" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B13" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C13" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C14" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B15" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C15" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B16" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C16" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C17" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C18" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B19" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C19" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B20" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C20" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B21" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C21" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B22" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C22" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B23" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C23" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B24" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C24" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B25" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C25" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B27" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C27" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B28" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C28" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
   </sheetData>

</xml_diff>